<commit_message>
updated podium for 25 april
</commit_message>
<xml_diff>
--- a/podium.xlsx
+++ b/podium.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7652" uniqueCount="708">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7659" uniqueCount="708">
   <si>
     <t xml:space="preserve">Magnum</t>
   </si>
@@ -2237,12 +2237,12 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -2434,7 +2434,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B7:AA1132"/>
+  <dimension ref="B7:AA1135"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27951,13 +27951,13 @@
         <v>8772</v>
       </c>
       <c r="O1120" s="3"/>
-      <c r="P1120" s="5" t="n">
+      <c r="P1120" s="3" t="n">
         <v>9933</v>
       </c>
-      <c r="Q1120" s="5" t="n">
+      <c r="Q1120" s="3" t="n">
         <v>6320</v>
       </c>
-      <c r="R1120" s="5" t="n">
+      <c r="R1120" s="3" t="n">
         <v>9432</v>
       </c>
       <c r="S1120" s="3"/>
@@ -27992,13 +27992,13 @@
         <v>7753</v>
       </c>
       <c r="O1121" s="3"/>
-      <c r="P1121" s="5" t="n">
+      <c r="P1121" s="3" t="n">
         <v>3221</v>
       </c>
-      <c r="Q1121" s="5" t="n">
+      <c r="Q1121" s="3" t="n">
         <v>9530</v>
       </c>
-      <c r="R1121" s="5" t="n">
+      <c r="R1121" s="3" t="n">
         <v>9652</v>
       </c>
       <c r="S1121" s="3"/>
@@ -28033,13 +28033,13 @@
         <v>8420</v>
       </c>
       <c r="O1122" s="3"/>
-      <c r="P1122" s="5" t="n">
+      <c r="P1122" s="3" t="n">
         <v>7641</v>
       </c>
-      <c r="Q1122" s="5" t="n">
+      <c r="Q1122" s="3" t="n">
         <v>6300</v>
       </c>
-      <c r="R1122" s="5" t="n">
+      <c r="R1122" s="3" t="n">
         <v>5420</v>
       </c>
       <c r="S1122" s="3"/>
@@ -28074,13 +28074,13 @@
         <v>9764</v>
       </c>
       <c r="O1123" s="3"/>
-      <c r="P1123" s="5" t="n">
+      <c r="P1123" s="3" t="n">
         <v>6520</v>
       </c>
-      <c r="Q1123" s="5" t="n">
+      <c r="Q1123" s="3" t="n">
         <v>6522</v>
       </c>
-      <c r="R1123" s="5" t="n">
+      <c r="R1123" s="3" t="n">
         <v>9970</v>
       </c>
       <c r="S1123" s="3"/>
@@ -28115,13 +28115,13 @@
         <v>8543</v>
       </c>
       <c r="O1124" s="3"/>
-      <c r="P1124" s="5" t="n">
+      <c r="P1124" s="3" t="n">
         <v>9942</v>
       </c>
-      <c r="Q1124" s="5" t="n">
+      <c r="Q1124" s="3" t="n">
         <v>8443</v>
       </c>
-      <c r="R1124" s="5" t="n">
+      <c r="R1124" s="3" t="n">
         <v>8854</v>
       </c>
       <c r="S1124" s="3"/>
@@ -28156,13 +28156,13 @@
         <v>5441</v>
       </c>
       <c r="O1125" s="3"/>
-      <c r="P1125" s="5" t="n">
+      <c r="P1125" s="3" t="n">
         <v>9721</v>
       </c>
-      <c r="Q1125" s="5" t="n">
+      <c r="Q1125" s="3" t="n">
         <v>8873</v>
       </c>
-      <c r="R1125" s="5" t="n">
+      <c r="R1125" s="3" t="n">
         <v>9732</v>
       </c>
       <c r="S1125" s="3"/>
@@ -28197,13 +28197,13 @@
         <v>9210</v>
       </c>
       <c r="O1126" s="3"/>
-      <c r="P1126" s="5" t="n">
+      <c r="P1126" s="3" t="n">
         <v>9766</v>
       </c>
-      <c r="Q1126" s="5" t="n">
+      <c r="Q1126" s="3" t="n">
         <v>9864</v>
       </c>
-      <c r="R1126" s="5" t="n">
+      <c r="R1126" s="3" t="n">
         <v>9332</v>
       </c>
       <c r="S1126" s="3"/>
@@ -28251,13 +28251,22 @@
       <c r="U1128" s="3"/>
     </row>
     <row r="1129" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C1129" s="1" t="s">
+        <v>0</v>
+      </c>
       <c r="D1129" s="3"/>
       <c r="E1129" s="3"/>
       <c r="F1129" s="3"/>
       <c r="G1129" s="3"/>
-      <c r="H1129" s="3"/>
-      <c r="I1129" s="3"/>
-      <c r="J1129" s="3"/>
+      <c r="H1129" s="3" t="n">
+        <v>7320</v>
+      </c>
+      <c r="I1129" s="3" t="n">
+        <v>9860</v>
+      </c>
+      <c r="J1129" s="3" t="n">
+        <v>5421</v>
+      </c>
       <c r="K1129" s="3"/>
       <c r="L1129" s="3"/>
       <c r="M1129" s="3"/>
@@ -28270,13 +28279,91 @@
       <c r="T1129" s="4"/>
     </row>
     <row r="1130" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C1130" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1130" s="5" t="n">
+        <v>9951</v>
+      </c>
+      <c r="I1130" s="5" t="n">
+        <v>5543</v>
+      </c>
+      <c r="J1130" s="5" t="n">
+        <v>9998</v>
+      </c>
       <c r="T1130" s="4"/>
     </row>
     <row r="1131" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C1131" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H1131" s="5" t="n">
+        <v>7754</v>
+      </c>
+      <c r="I1131" s="5" t="n">
+        <v>9652</v>
+      </c>
+      <c r="J1131" s="5" t="n">
+        <v>7622</v>
+      </c>
       <c r="T1131" s="4"/>
     </row>
     <row r="1132" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C1132" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1132" s="5" t="n">
+        <v>8510</v>
+      </c>
+      <c r="I1132" s="5" t="n">
+        <v>8432</v>
+      </c>
+      <c r="J1132" s="5" t="n">
+        <v>8861</v>
+      </c>
       <c r="T1132" s="4"/>
+    </row>
+    <row r="1133" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C1133" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1133" s="5" t="n">
+        <v>9652</v>
+      </c>
+      <c r="I1133" s="5" t="n">
+        <v>8510</v>
+      </c>
+      <c r="J1133" s="5" t="n">
+        <v>8632</v>
+      </c>
+    </row>
+    <row r="1134" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C1134" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="H1134" s="5" t="n">
+        <v>9950</v>
+      </c>
+      <c r="I1134" s="5" t="n">
+        <v>6000</v>
+      </c>
+      <c r="J1134" s="5" t="n">
+        <v>9760</v>
+      </c>
+    </row>
+    <row r="1135" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C1135" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="H1135" s="5" t="n">
+        <v>2211</v>
+      </c>
+      <c r="I1135" s="5" t="n">
+        <v>9500</v>
+      </c>
+      <c r="J1135" s="5" t="n">
+        <v>5550</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
updated podium for 29 april
</commit_message>
<xml_diff>
--- a/podium.xlsx
+++ b/podium.xlsx
@@ -2220,7 +2220,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2239,6 +2239,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -28264,9 +28268,15 @@
         <v>5421</v>
       </c>
       <c r="K1129" s="3"/>
-      <c r="L1129" s="3"/>
-      <c r="M1129" s="3"/>
-      <c r="N1129" s="3"/>
+      <c r="L1129" s="3" t="n">
+        <v>6320</v>
+      </c>
+      <c r="M1129" s="3" t="n">
+        <v>9830</v>
+      </c>
+      <c r="N1129" s="3" t="n">
+        <v>8554</v>
+      </c>
       <c r="O1129" s="3"/>
       <c r="P1129" s="3"/>
       <c r="Q1129" s="3"/>
@@ -28287,6 +28297,15 @@
       <c r="J1130" s="3" t="n">
         <v>9998</v>
       </c>
+      <c r="L1130" s="5" t="n">
+        <v>8443</v>
+      </c>
+      <c r="M1130" s="5" t="n">
+        <v>7431</v>
+      </c>
+      <c r="N1130" s="5" t="n">
+        <v>9853</v>
+      </c>
       <c r="T1130" s="4"/>
     </row>
     <row r="1131" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28302,6 +28321,15 @@
       <c r="J1131" s="3" t="n">
         <v>7622</v>
       </c>
+      <c r="L1131" s="5" t="n">
+        <v>7320</v>
+      </c>
+      <c r="M1131" s="5" t="n">
+        <v>9541</v>
+      </c>
+      <c r="N1131" s="5" t="n">
+        <v>7622</v>
+      </c>
       <c r="T1131" s="4"/>
     </row>
     <row r="1132" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28317,6 +28345,15 @@
       <c r="J1132" s="3" t="n">
         <v>8861</v>
       </c>
+      <c r="L1132" s="5" t="n">
+        <v>7320</v>
+      </c>
+      <c r="M1132" s="5" t="n">
+        <v>9310</v>
+      </c>
+      <c r="N1132" s="5" t="n">
+        <v>6543</v>
+      </c>
       <c r="T1132" s="4"/>
     </row>
     <row r="1133" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28332,6 +28369,15 @@
       <c r="J1133" s="3" t="n">
         <v>8632</v>
       </c>
+      <c r="L1133" s="5" t="n">
+        <v>8632</v>
+      </c>
+      <c r="M1133" s="5" t="n">
+        <v>6651</v>
+      </c>
+      <c r="N1133" s="5" t="n">
+        <v>3221</v>
+      </c>
     </row>
     <row r="1134" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C1134" s="1" t="s">
@@ -28346,6 +28392,15 @@
       <c r="J1134" s="3" t="n">
         <v>9760</v>
       </c>
+      <c r="L1134" s="5" t="n">
+        <v>7611</v>
+      </c>
+      <c r="M1134" s="5" t="n">
+        <v>9752</v>
+      </c>
+      <c r="N1134" s="5" t="n">
+        <v>8644</v>
+      </c>
     </row>
     <row r="1135" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C1135" s="1" t="s">
@@ -28359,6 +28414,15 @@
       </c>
       <c r="J1135" s="3" t="n">
         <v>5550</v>
+      </c>
+      <c r="L1135" s="5" t="n">
+        <v>7542</v>
+      </c>
+      <c r="M1135" s="5" t="n">
+        <v>8741</v>
+      </c>
+      <c r="N1135" s="5" t="n">
+        <v>3221</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor main.py into modular step-based architecture
</commit_message>
<xml_diff>
--- a/podium.xlsx
+++ b/podium.xlsx
@@ -2242,7 +2242,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -27923,7 +27923,7 @@
       <c r="T1119" s="4"/>
       <c r="U1119" s="3"/>
     </row>
-    <row r="1120" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1120" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C1120" s="1" t="s">
         <v>0</v>
       </c>
@@ -27962,9 +27962,9 @@
       </c>
       <c r="S1120" s="3"/>
       <c r="T1120" s="4"/>
-      <c r="U1120" s="3"/>
-    </row>
-    <row r="1121" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="U1120" s="5"/>
+    </row>
+    <row r="1121" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C1121" s="1" t="s">
         <v>10</v>
       </c>
@@ -28003,9 +28003,9 @@
       </c>
       <c r="S1121" s="3"/>
       <c r="T1121" s="4"/>
-      <c r="U1121" s="3"/>
-    </row>
-    <row r="1122" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="U1121" s="5"/>
+    </row>
+    <row r="1122" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C1122" s="1" t="s">
         <v>20</v>
       </c>
@@ -28044,9 +28044,9 @@
       </c>
       <c r="S1122" s="3"/>
       <c r="T1122" s="4"/>
-      <c r="U1122" s="3"/>
-    </row>
-    <row r="1123" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="U1122" s="5"/>
+    </row>
+    <row r="1123" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C1123" s="1" t="s">
         <v>30</v>
       </c>
@@ -28085,7 +28085,7 @@
       </c>
       <c r="S1123" s="3"/>
       <c r="T1123" s="4"/>
-      <c r="U1123" s="3"/>
+      <c r="U1123" s="5"/>
     </row>
     <row r="1124" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C1124" s="1" t="s">
@@ -28126,7 +28126,7 @@
       </c>
       <c r="S1124" s="3"/>
       <c r="T1124" s="4"/>
-      <c r="U1124" s="3"/>
+      <c r="U1124" s="5"/>
     </row>
     <row r="1125" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C1125" s="1" t="s">
@@ -28167,7 +28167,7 @@
       </c>
       <c r="S1125" s="3"/>
       <c r="T1125" s="4"/>
-      <c r="U1125" s="3"/>
+      <c r="U1125" s="5"/>
     </row>
     <row r="1126" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C1126" s="1" t="s">
@@ -28208,7 +28208,7 @@
       </c>
       <c r="S1126" s="3"/>
       <c r="T1126" s="4"/>
-      <c r="U1126" s="3"/>
+      <c r="U1126" s="5"/>
     </row>
     <row r="1127" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D1127" s="3"/>
@@ -28228,7 +28228,7 @@
       <c r="R1127" s="3"/>
       <c r="S1127" s="3"/>
       <c r="T1127" s="4"/>
-      <c r="U1127" s="3"/>
+      <c r="U1127" s="5"/>
     </row>
     <row r="1128" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D1128" s="3"/>
@@ -28248,7 +28248,7 @@
       <c r="R1128" s="3"/>
       <c r="S1128" s="3"/>
       <c r="T1128" s="4"/>
-      <c r="U1128" s="3"/>
+      <c r="U1128" s="5"/>
     </row>
     <row r="1129" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C1129" s="1" t="s">
@@ -28283,6 +28283,7 @@
       <c r="R1129" s="3"/>
       <c r="S1129" s="3"/>
       <c r="T1129" s="4"/>
+      <c r="U1129" s="5"/>
     </row>
     <row r="1130" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C1130" s="1" t="s">
@@ -28297,16 +28298,17 @@
       <c r="J1130" s="3" t="n">
         <v>9998</v>
       </c>
-      <c r="L1130" s="5" t="n">
+      <c r="L1130" s="3" t="n">
         <v>8443</v>
       </c>
-      <c r="M1130" s="5" t="n">
+      <c r="M1130" s="3" t="n">
         <v>7431</v>
       </c>
-      <c r="N1130" s="5" t="n">
+      <c r="N1130" s="3" t="n">
         <v>9853</v>
       </c>
       <c r="T1130" s="4"/>
+      <c r="U1130" s="5"/>
     </row>
     <row r="1131" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C1131" s="1" t="s">
@@ -28321,16 +28323,17 @@
       <c r="J1131" s="3" t="n">
         <v>7622</v>
       </c>
-      <c r="L1131" s="5" t="n">
+      <c r="L1131" s="3" t="n">
         <v>7320</v>
       </c>
-      <c r="M1131" s="5" t="n">
+      <c r="M1131" s="3" t="n">
         <v>9541</v>
       </c>
-      <c r="N1131" s="5" t="n">
+      <c r="N1131" s="3" t="n">
         <v>7622</v>
       </c>
       <c r="T1131" s="4"/>
+      <c r="U1131" s="5"/>
     </row>
     <row r="1132" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C1132" s="1" t="s">
@@ -28345,16 +28348,17 @@
       <c r="J1132" s="3" t="n">
         <v>8861</v>
       </c>
-      <c r="L1132" s="5" t="n">
+      <c r="L1132" s="3" t="n">
         <v>7320</v>
       </c>
-      <c r="M1132" s="5" t="n">
+      <c r="M1132" s="3" t="n">
         <v>9310</v>
       </c>
-      <c r="N1132" s="5" t="n">
+      <c r="N1132" s="3" t="n">
         <v>6543</v>
       </c>
       <c r="T1132" s="4"/>
+      <c r="U1132" s="5"/>
     </row>
     <row r="1133" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C1133" s="1" t="s">
@@ -28369,15 +28373,16 @@
       <c r="J1133" s="3" t="n">
         <v>8632</v>
       </c>
-      <c r="L1133" s="5" t="n">
+      <c r="L1133" s="3" t="n">
         <v>8632</v>
       </c>
-      <c r="M1133" s="5" t="n">
+      <c r="M1133" s="3" t="n">
         <v>6651</v>
       </c>
-      <c r="N1133" s="5" t="n">
+      <c r="N1133" s="3" t="n">
         <v>3221</v>
       </c>
+      <c r="U1133" s="5"/>
     </row>
     <row r="1134" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C1134" s="1" t="s">
@@ -28392,15 +28397,16 @@
       <c r="J1134" s="3" t="n">
         <v>9760</v>
       </c>
-      <c r="L1134" s="5" t="n">
+      <c r="L1134" s="3" t="n">
         <v>7611</v>
       </c>
-      <c r="M1134" s="5" t="n">
+      <c r="M1134" s="3" t="n">
         <v>9752</v>
       </c>
-      <c r="N1134" s="5" t="n">
+      <c r="N1134" s="3" t="n">
         <v>8644</v>
       </c>
+      <c r="U1134" s="5"/>
     </row>
     <row r="1135" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C1135" s="1" t="s">
@@ -28415,15 +28421,16 @@
       <c r="J1135" s="3" t="n">
         <v>5550</v>
       </c>
-      <c r="L1135" s="5" t="n">
+      <c r="L1135" s="3" t="n">
         <v>7542</v>
       </c>
-      <c r="M1135" s="5" t="n">
+      <c r="M1135" s="3" t="n">
         <v>8741</v>
       </c>
-      <c r="N1135" s="5" t="n">
+      <c r="N1135" s="3" t="n">
         <v>3221</v>
       </c>
+      <c r="U1135" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>